<commit_message>
added new styling to the dashboard
</commit_message>
<xml_diff>
--- a/data/data_records.xlsx
+++ b/data/data_records.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gpain/Documents/Work_Dashboards/Arizona/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{194DA4E3-D321-BD4B-9F87-E3C1395E3D7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D4DB03-8A7E-2644-94CA-02A7103CC8D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="0" windowWidth="51200" windowHeight="28800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Organizations" sheetId="1" r:id="rId1"/>
@@ -6506,7 +6506,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6561,8 +6561,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -6570,7 +6568,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -6814,9 +6812,9 @@
   <dimension ref="A1:V91"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="43.1640625" style="25" customWidth="1"/>
+    <col min="1" max="1" width="43.1640625" style="23" customWidth="1"/>
     <col min="2" max="2" width="50.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="59.1640625" style="23" customWidth="1"/>
+    <col min="3" max="3" width="59.1640625" customWidth="1"/>
     <col min="4" max="4" width="40.6640625" customWidth="1"/>
     <col min="5" max="5" width="29.1640625" customWidth="1"/>
     <col min="6" max="6" width="5.33203125" bestFit="1" customWidth="1"/>
@@ -6824,16 +6822,16 @@
     <col min="8" max="8" width="13.33203125" customWidth="1"/>
     <col min="9" max="9" width="16.33203125" customWidth="1"/>
     <col min="10" max="10" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="40" style="25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="36.83203125" style="25" customWidth="1"/>
+    <col min="11" max="11" width="40" style="23" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="36.83203125" style="23" customWidth="1"/>
     <col min="13" max="13" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="29.83203125" style="25" customWidth="1"/>
-    <col min="15" max="15" width="30" style="25" customWidth="1"/>
-    <col min="16" max="16" width="39.83203125" style="25" customWidth="1"/>
-    <col min="17" max="17" width="28.5" style="25" customWidth="1"/>
-    <col min="18" max="18" width="61" style="25" customWidth="1"/>
-    <col min="19" max="19" width="32.33203125" style="25" customWidth="1"/>
-    <col min="20" max="20" width="38.1640625" style="25" customWidth="1"/>
+    <col min="14" max="14" width="29.83203125" style="23" customWidth="1"/>
+    <col min="15" max="15" width="30" style="23" customWidth="1"/>
+    <col min="16" max="16" width="39.83203125" style="23" customWidth="1"/>
+    <col min="17" max="17" width="28.5" style="23" customWidth="1"/>
+    <col min="18" max="18" width="61" style="23" customWidth="1"/>
+    <col min="19" max="19" width="32.33203125" style="23" customWidth="1"/>
+    <col min="20" max="20" width="38.1640625" style="23" customWidth="1"/>
     <col min="21" max="21" width="26.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6841,13 +6839,13 @@
       <c r="A1" s="1" t="s">
         <v>1149</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="24" t="s">
         <v>1150</v>
       </c>
       <c r="C1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="24" t="s">
         <v>1153</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -6856,7 +6854,7 @@
       <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="26" t="s">
+      <c r="G1" s="24" t="s">
         <v>1152</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -6865,43 +6863,43 @@
       <c r="I1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="26" t="s">
+      <c r="J1" s="24" t="s">
         <v>1151</v>
       </c>
-      <c r="K1" s="26" t="s">
+      <c r="K1" s="24" t="s">
         <v>1155</v>
       </c>
-      <c r="L1" s="26" t="s">
+      <c r="L1" s="24" t="s">
         <v>1156</v>
       </c>
-      <c r="M1" s="26" t="s">
+      <c r="M1" s="24" t="s">
         <v>1172</v>
       </c>
-      <c r="N1" s="35" t="s">
+      <c r="N1" s="33" t="s">
         <v>1169</v>
       </c>
-      <c r="O1" s="26" t="s">
+      <c r="O1" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="26" t="s">
+      <c r="P1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="Q1" s="26" t="s">
+      <c r="Q1" s="24" t="s">
         <v>1170</v>
       </c>
-      <c r="R1" s="26" t="s">
+      <c r="R1" s="24" t="s">
         <v>1173</v>
       </c>
-      <c r="S1" s="26" t="s">
+      <c r="S1" s="24" t="s">
         <v>1163</v>
       </c>
-      <c r="T1" s="26" t="s">
+      <c r="T1" s="24" t="s">
         <v>1164</v>
       </c>
-      <c r="U1" s="26" t="s">
+      <c r="U1" s="24" t="s">
         <v>1157</v>
       </c>
-      <c r="V1" s="26" t="s">
+      <c r="V1" s="24" t="s">
         <v>1171</v>
       </c>
     </row>
@@ -6912,7 +6910,7 @@
       <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="25" t="s">
         <v>9</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -6946,7 +6944,7 @@
         <v>12500</v>
       </c>
       <c r="N2" s="19"/>
-      <c r="O2" s="29">
+      <c r="O2" s="27">
         <v>0</v>
       </c>
       <c r="P2" s="19"/>
@@ -6969,7 +6967,7 @@
       <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" s="25" t="s">
         <v>19</v>
       </c>
       <c r="D3" s="5" t="s">
@@ -7020,7 +7018,7 @@
       <c r="B4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="25" t="s">
         <v>25</v>
       </c>
       <c r="D4" s="5" t="s">
@@ -7071,7 +7069,7 @@
       <c r="B5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="25" t="s">
         <v>33</v>
       </c>
       <c r="D5" s="3" t="s">
@@ -7103,7 +7101,7 @@
       </c>
       <c r="M5" s="5"/>
       <c r="N5" s="19"/>
-      <c r="O5" s="29">
+      <c r="O5" s="27">
         <v>0</v>
       </c>
       <c r="P5" s="19"/>
@@ -7128,7 +7126,7 @@
       <c r="B6" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="27" t="s">
+      <c r="C6" s="25" t="s">
         <v>39</v>
       </c>
       <c r="D6" s="5" t="s">
@@ -7179,7 +7177,7 @@
       <c r="B7" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="27" t="s">
+      <c r="C7" s="25" t="s">
         <v>44</v>
       </c>
       <c r="D7" s="5" t="s">
@@ -7211,7 +7209,7 @@
       </c>
       <c r="M7" s="5"/>
       <c r="N7" s="19"/>
-      <c r="O7" s="30">
+      <c r="O7" s="28">
         <v>0</v>
       </c>
       <c r="P7" s="19"/>
@@ -7232,7 +7230,7 @@
       <c r="B8" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="25" t="s">
         <v>49</v>
       </c>
       <c r="D8" s="5" t="s">
@@ -7285,7 +7283,7 @@
       <c r="B9" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="25" t="s">
         <v>55</v>
       </c>
       <c r="D9" s="5" t="s">
@@ -7342,7 +7340,7 @@
       <c r="B10" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="27" t="s">
+      <c r="C10" s="25" t="s">
         <v>62</v>
       </c>
       <c r="D10" s="5" t="s">
@@ -7393,7 +7391,7 @@
       <c r="B11" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="27" t="s">
+      <c r="C11" s="25" t="s">
         <v>66</v>
       </c>
       <c r="D11" s="5" t="s">
@@ -7444,7 +7442,7 @@
       <c r="B12" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C12" s="27" t="s">
+      <c r="C12" s="25" t="s">
         <v>71</v>
       </c>
       <c r="D12" s="5" t="s">
@@ -7495,7 +7493,7 @@
       <c r="B13" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="27" t="s">
+      <c r="C13" s="25" t="s">
         <v>75</v>
       </c>
       <c r="D13" s="5" t="s">
@@ -7546,7 +7544,7 @@
       <c r="B14" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="25" t="s">
         <v>78</v>
       </c>
       <c r="D14" s="5" t="s">
@@ -7605,7 +7603,7 @@
       <c r="B15" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="27" t="s">
+      <c r="C15" s="25" t="s">
         <v>87</v>
       </c>
       <c r="D15" s="5" t="s">
@@ -7656,7 +7654,7 @@
       <c r="B16" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="27" t="s">
+      <c r="C16" s="25" t="s">
         <v>90</v>
       </c>
       <c r="D16" s="3" t="s">
@@ -7713,7 +7711,7 @@
       <c r="B17" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="25" t="s">
         <v>97</v>
       </c>
       <c r="D17" s="3" t="s">
@@ -7770,7 +7768,7 @@
       <c r="B18" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="27" t="s">
+      <c r="C18" s="25" t="s">
         <v>102</v>
       </c>
       <c r="D18" s="5" t="s">
@@ -7821,7 +7819,7 @@
       <c r="B19" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="27" t="s">
+      <c r="C19" s="25" t="s">
         <v>105</v>
       </c>
       <c r="D19" s="5" t="s">
@@ -7872,7 +7870,7 @@
       <c r="B20" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C20" s="27" t="s">
+      <c r="C20" s="25" t="s">
         <v>109</v>
       </c>
       <c r="D20" s="5" t="s">
@@ -7923,7 +7921,7 @@
       <c r="B21" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="27" t="s">
+      <c r="C21" s="25" t="s">
         <v>113</v>
       </c>
       <c r="D21" s="3" t="s">
@@ -7967,14 +7965,14 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:21" ht="28">
+    <row r="22" spans="1:21" ht="14">
       <c r="A22" s="19" t="s">
         <v>117</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C22" s="27" t="s">
+      <c r="C22" s="25" t="s">
         <v>118</v>
       </c>
       <c r="D22" s="5" t="s">
@@ -8022,14 +8020,14 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="140">
+    <row r="23" spans="1:21" ht="112">
       <c r="A23" s="19" t="s">
         <v>123</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="22"/>
+      <c r="C23" s="5"/>
       <c r="D23" s="5"/>
       <c r="E23" s="5" t="s">
         <v>124</v>
@@ -8059,7 +8057,7 @@
         <v>50</v>
       </c>
       <c r="N23" s="19"/>
-      <c r="O23" s="31">
+      <c r="O23" s="29">
         <v>0</v>
       </c>
       <c r="P23" s="19"/>
@@ -8084,7 +8082,7 @@
       <c r="B24" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C24" s="27" t="s">
+      <c r="C24" s="25" t="s">
         <v>130</v>
       </c>
       <c r="D24" s="5" t="s">
@@ -8137,7 +8135,7 @@
       <c r="B25" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C25" s="27" t="s">
+      <c r="C25" s="25" t="s">
         <v>133</v>
       </c>
       <c r="D25" s="5" t="s">
@@ -8200,7 +8198,7 @@
       <c r="B26" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C26" s="27" t="s">
+      <c r="C26" s="25" t="s">
         <v>144</v>
       </c>
       <c r="D26" s="5" t="s">
@@ -8255,7 +8253,7 @@
       <c r="B27" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C27" s="27" t="s">
+      <c r="C27" s="25" t="s">
         <v>149</v>
       </c>
       <c r="D27" s="5" t="s">
@@ -8291,7 +8289,7 @@
       <c r="N27" s="19" t="s">
         <v>152</v>
       </c>
-      <c r="O27" s="29">
+      <c r="O27" s="27">
         <v>0</v>
       </c>
       <c r="P27" s="19" t="s">
@@ -8318,7 +8316,7 @@
       <c r="B28" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="27" t="s">
+      <c r="C28" s="25" t="s">
         <v>158</v>
       </c>
       <c r="D28" s="3" t="s">
@@ -8354,7 +8352,7 @@
       <c r="N28" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="O28" s="30">
+      <c r="O28" s="28">
         <v>0</v>
       </c>
       <c r="P28" s="18" t="s">
@@ -8381,7 +8379,7 @@
       <c r="B29" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C29" s="27" t="s">
+      <c r="C29" s="25" t="s">
         <v>167</v>
       </c>
       <c r="D29" s="3" t="s">
@@ -8434,7 +8432,7 @@
       <c r="B30" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C30" s="27" t="s">
+      <c r="C30" s="25" t="s">
         <v>173</v>
       </c>
       <c r="D30" s="3" t="s">
@@ -8489,7 +8487,7 @@
       <c r="B31" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C31" s="27" t="s">
+      <c r="C31" s="25" t="s">
         <v>178</v>
       </c>
       <c r="D31" s="5" t="s">
@@ -8550,7 +8548,7 @@
       <c r="B32" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C32" s="27" t="s">
+      <c r="C32" s="25" t="s">
         <v>186</v>
       </c>
       <c r="D32" s="5" t="s">
@@ -8601,7 +8599,7 @@
       <c r="B33" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="C33" s="27" t="s">
+      <c r="C33" s="25" t="s">
         <v>191</v>
       </c>
       <c r="D33" s="5" t="s">
@@ -8652,7 +8650,7 @@
       <c r="B34" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C34" s="27" t="s">
+      <c r="C34" s="25" t="s">
         <v>194</v>
       </c>
       <c r="D34" s="5"/>
@@ -8711,7 +8709,7 @@
       <c r="B35" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C35" s="27" t="s">
+      <c r="C35" s="25" t="s">
         <v>200</v>
       </c>
       <c r="D35" s="3" t="s">
@@ -8745,7 +8743,7 @@
         <v>10000</v>
       </c>
       <c r="N35" s="18"/>
-      <c r="O35" s="30">
+      <c r="O35" s="28">
         <v>0</v>
       </c>
       <c r="P35" s="18" t="s">
@@ -8766,13 +8764,13 @@
       </c>
     </row>
     <row r="36" spans="1:21" ht="56">
-      <c r="A36" s="24" t="s">
+      <c r="A36" s="22" t="s">
         <v>206</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="C36" s="27" t="s">
+      <c r="C36" s="25" t="s">
         <v>207</v>
       </c>
       <c r="D36" s="3" t="s">
@@ -8804,7 +8802,7 @@
       </c>
       <c r="M36" s="3"/>
       <c r="N36" s="18"/>
-      <c r="O36" s="30">
+      <c r="O36" s="28">
         <v>0</v>
       </c>
       <c r="P36" s="18" t="s">
@@ -8829,7 +8827,7 @@
       <c r="B37" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C37" s="27" t="s">
+      <c r="C37" s="25" t="s">
         <v>213</v>
       </c>
       <c r="D37" s="5" t="s">
@@ -8875,14 +8873,14 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:21" ht="42">
+    <row r="38" spans="1:21" ht="28">
       <c r="A38" s="19" t="s">
         <v>216</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C38" s="27" t="s">
+      <c r="C38" s="25" t="s">
         <v>217</v>
       </c>
       <c r="D38" s="5" t="s">
@@ -8939,7 +8937,7 @@
       <c r="B39" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C39" s="27" t="s">
+      <c r="C39" s="25" t="s">
         <v>223</v>
       </c>
       <c r="D39" s="12" t="s">
@@ -8989,14 +8987,14 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:21" ht="168">
+    <row r="40" spans="1:21" ht="126">
       <c r="A40" s="19" t="s">
         <v>227</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C40" s="27" t="s">
+      <c r="C40" s="25" t="s">
         <v>228</v>
       </c>
       <c r="D40" s="5" t="s">
@@ -9059,7 +9057,7 @@
       <c r="B41" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C41" s="27" t="s">
+      <c r="C41" s="25" t="s">
         <v>237</v>
       </c>
       <c r="D41" s="5"/>
@@ -9108,7 +9106,7 @@
       <c r="B42" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C42" s="27" t="s">
+      <c r="C42" s="25" t="s">
         <v>240</v>
       </c>
       <c r="D42" s="5" t="s">
@@ -9144,7 +9142,7 @@
       <c r="N42" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="O42" s="29">
+      <c r="O42" s="27">
         <v>0</v>
       </c>
       <c r="P42" s="19" t="s">
@@ -9173,7 +9171,7 @@
       <c r="B43" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C43" s="27" t="s">
+      <c r="C43" s="25" t="s">
         <v>251</v>
       </c>
       <c r="D43" s="5" t="s">
@@ -9228,7 +9226,7 @@
       <c r="B44" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="C44" s="27" t="s">
+      <c r="C44" s="25" t="s">
         <v>256</v>
       </c>
       <c r="D44" s="5" t="s">
@@ -9279,7 +9277,7 @@
       <c r="B45" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C45" s="27" t="s">
+      <c r="C45" s="25" t="s">
         <v>259</v>
       </c>
       <c r="D45" s="5" t="s">
@@ -9311,7 +9309,7 @@
       </c>
       <c r="M45" s="5"/>
       <c r="N45" s="19"/>
-      <c r="O45" s="30">
+      <c r="O45" s="28">
         <v>0</v>
       </c>
       <c r="P45" s="19"/>
@@ -9332,7 +9330,7 @@
       <c r="B46" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C46" s="27" t="s">
+      <c r="C46" s="25" t="s">
         <v>262</v>
       </c>
       <c r="D46" s="5" t="s">
@@ -9366,7 +9364,7 @@
         <v>20000</v>
       </c>
       <c r="N46" s="19"/>
-      <c r="O46" s="30">
+      <c r="O46" s="28">
         <v>0</v>
       </c>
       <c r="P46" s="19" t="s">
@@ -9393,7 +9391,7 @@
       <c r="B47" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C47" s="27" t="s">
+      <c r="C47" s="25" t="s">
         <v>269</v>
       </c>
       <c r="D47" s="5" t="s">
@@ -9446,7 +9444,7 @@
       <c r="B48" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C48" s="27" t="s">
+      <c r="C48" s="25" t="s">
         <v>274</v>
       </c>
       <c r="D48" s="5" t="s">
@@ -9492,14 +9490,14 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:21" ht="70">
+    <row r="49" spans="1:21" ht="42">
       <c r="A49" s="19" t="s">
         <v>277</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C49" s="27" t="s">
+      <c r="C49" s="25" t="s">
         <v>278</v>
       </c>
       <c r="D49" s="5" t="s">
@@ -9531,7 +9529,7 @@
       </c>
       <c r="M49" s="5"/>
       <c r="N49" s="19"/>
-      <c r="O49" s="30">
+      <c r="O49" s="28">
         <v>0</v>
       </c>
       <c r="P49" s="19"/>
@@ -9554,7 +9552,7 @@
       <c r="B50" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="C50" s="27" t="s">
+      <c r="C50" s="25" t="s">
         <v>282</v>
       </c>
       <c r="D50" s="5" t="s">
@@ -9617,7 +9615,7 @@
       <c r="B51" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C51" s="27" t="s">
+      <c r="C51" s="25" t="s">
         <v>291</v>
       </c>
       <c r="D51" s="5"/>
@@ -9668,7 +9666,7 @@
       <c r="B52" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C52" s="27" t="s">
+      <c r="C52" s="25" t="s">
         <v>294</v>
       </c>
       <c r="D52" s="5" t="s">
@@ -9719,7 +9717,7 @@
       <c r="B53" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C53" s="27" t="s">
+      <c r="C53" s="25" t="s">
         <v>297</v>
       </c>
       <c r="D53" s="5"/>
@@ -9768,7 +9766,7 @@
       <c r="B54" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C54" s="27" t="s">
+      <c r="C54" s="25" t="s">
         <v>299</v>
       </c>
       <c r="D54" s="5"/>
@@ -9827,7 +9825,7 @@
       <c r="B55" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C55" s="27" t="s">
+      <c r="C55" s="25" t="s">
         <v>306</v>
       </c>
       <c r="D55" s="5" t="s">
@@ -9880,7 +9878,7 @@
       <c r="B56" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C56" s="27" t="s">
+      <c r="C56" s="25" t="s">
         <v>310</v>
       </c>
       <c r="D56" s="5" t="s">
@@ -9931,7 +9929,7 @@
       <c r="B57" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C57" s="27" t="s">
+      <c r="C57" s="25" t="s">
         <v>314</v>
       </c>
       <c r="D57" s="3"/>
@@ -9982,7 +9980,7 @@
       <c r="B58" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C58" s="27" t="s">
+      <c r="C58" s="25" t="s">
         <v>317</v>
       </c>
       <c r="D58" s="3" t="s">
@@ -10033,7 +10031,7 @@
       <c r="B59" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C59" s="27" t="s">
+      <c r="C59" s="25" t="s">
         <v>320</v>
       </c>
       <c r="D59" s="3" t="s">
@@ -10083,14 +10081,14 @@
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:21" ht="42">
+    <row r="60" spans="1:21" ht="28">
       <c r="A60" s="19" t="s">
         <v>325</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C60" s="27" t="s">
+      <c r="C60" s="25" t="s">
         <v>326</v>
       </c>
       <c r="D60" s="5" t="s">
@@ -10122,7 +10120,7 @@
       </c>
       <c r="M60" s="5"/>
       <c r="N60" s="19"/>
-      <c r="O60" s="29">
+      <c r="O60" s="27">
         <v>0</v>
       </c>
       <c r="P60" s="19"/>
@@ -10145,7 +10143,7 @@
       <c r="B61" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C61" s="27" t="s">
+      <c r="C61" s="25" t="s">
         <v>330</v>
       </c>
       <c r="D61" s="3" t="s">
@@ -10196,7 +10194,7 @@
       <c r="B62" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C62" s="27" t="s">
+      <c r="C62" s="25" t="s">
         <v>333</v>
       </c>
       <c r="D62" s="5" t="s">
@@ -10247,7 +10245,7 @@
       <c r="B63" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C63" s="27" t="s">
+      <c r="C63" s="25" t="s">
         <v>336</v>
       </c>
       <c r="D63" s="5" t="s">
@@ -10298,7 +10296,7 @@
       <c r="B64" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C64" s="27" t="s">
+      <c r="C64" s="25" t="s">
         <v>339</v>
       </c>
       <c r="D64" s="5" t="s">
@@ -10351,7 +10349,7 @@
       <c r="B65" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C65" s="27" t="s">
+      <c r="C65" s="25" t="s">
         <v>343</v>
       </c>
       <c r="D65" s="5" t="s">
@@ -10387,7 +10385,7 @@
       <c r="N65" s="19" t="s">
         <v>346</v>
       </c>
-      <c r="O65" s="31">
+      <c r="O65" s="29">
         <v>0</v>
       </c>
       <c r="P65" s="19" t="s">
@@ -10414,7 +10412,7 @@
       <c r="B66" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C66" s="27" t="s">
+      <c r="C66" s="25" t="s">
         <v>351</v>
       </c>
       <c r="D66" s="5" t="s">
@@ -10467,7 +10465,7 @@
       <c r="B67" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C67" s="27" t="s">
+      <c r="C67" s="25" t="s">
         <v>355</v>
       </c>
       <c r="D67" s="5" t="s">
@@ -10520,7 +10518,7 @@
       <c r="B68" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C68" s="27" t="s">
+      <c r="C68" s="25" t="s">
         <v>359</v>
       </c>
       <c r="D68" s="5" t="s">
@@ -10573,7 +10571,7 @@
       <c r="B69" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="C69" s="27" t="s">
+      <c r="C69" s="25" t="s">
         <v>363</v>
       </c>
       <c r="D69" s="5" t="s">
@@ -10624,7 +10622,7 @@
       <c r="B70" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C70" s="27" t="s">
+      <c r="C70" s="25" t="s">
         <v>367</v>
       </c>
       <c r="D70" s="5" t="s">
@@ -10677,7 +10675,7 @@
       <c r="B71" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C71" s="27" t="s">
+      <c r="C71" s="25" t="s">
         <v>371</v>
       </c>
       <c r="D71" s="5" t="s">
@@ -10730,7 +10728,7 @@
       <c r="B72" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C72" s="27" t="s">
+      <c r="C72" s="25" t="s">
         <v>375</v>
       </c>
       <c r="D72" s="5"/>
@@ -10779,7 +10777,7 @@
       <c r="B73" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C73" s="27" t="s">
+      <c r="C73" s="25" t="s">
         <v>377</v>
       </c>
       <c r="D73" s="5" t="s">
@@ -10832,7 +10830,7 @@
       <c r="B74" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C74" s="27" t="s">
+      <c r="C74" s="25" t="s">
         <v>381</v>
       </c>
       <c r="D74" s="5" t="s">
@@ -10885,7 +10883,7 @@
       <c r="B75" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C75" s="27" t="s">
+      <c r="C75" s="25" t="s">
         <v>385</v>
       </c>
       <c r="D75" s="5"/>
@@ -10917,7 +10915,7 @@
         <v>15</v>
       </c>
       <c r="N75" s="19"/>
-      <c r="O75" s="31">
+      <c r="O75" s="29">
         <v>147</v>
       </c>
       <c r="P75" s="19"/>
@@ -10940,7 +10938,7 @@
       <c r="B76" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C76" s="27" t="s">
+      <c r="C76" s="25" t="s">
         <v>388</v>
       </c>
       <c r="D76" s="5" t="s">
@@ -10991,7 +10989,7 @@
       <c r="B77" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C77" s="27" t="s">
+      <c r="C77" s="25" t="s">
         <v>391</v>
       </c>
       <c r="D77" s="5" t="s">
@@ -11046,7 +11044,7 @@
       <c r="B78" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C78" s="27" t="s">
+      <c r="C78" s="25" t="s">
         <v>396</v>
       </c>
       <c r="D78" s="5" t="s">
@@ -11080,7 +11078,7 @@
         <v>200</v>
       </c>
       <c r="N78" s="19"/>
-      <c r="O78" s="29">
+      <c r="O78" s="27">
         <v>0</v>
       </c>
       <c r="P78" s="19" t="s">
@@ -11103,13 +11101,13 @@
       </c>
     </row>
     <row r="79" spans="1:21" ht="14">
-      <c r="A79" s="24" t="s">
+      <c r="A79" s="22" t="s">
         <v>401</v>
       </c>
       <c r="B79" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C79" s="27" t="s">
+      <c r="C79" s="25" t="s">
         <v>402</v>
       </c>
       <c r="D79" s="3" t="s">
@@ -11162,7 +11160,7 @@
       <c r="B80" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C80" s="27" t="s">
+      <c r="C80" s="25" t="s">
         <v>405</v>
       </c>
       <c r="D80" s="3" t="s">
@@ -11198,7 +11196,7 @@
       <c r="N80" s="18" t="s">
         <v>285</v>
       </c>
-      <c r="O80" s="30">
+      <c r="O80" s="28">
         <v>0</v>
       </c>
       <c r="P80" s="18" t="s">
@@ -11227,7 +11225,7 @@
       <c r="B81" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C81" s="27" t="s">
+      <c r="C81" s="25" t="s">
         <v>413</v>
       </c>
       <c r="D81" s="3" t="s">
@@ -11278,7 +11276,7 @@
       <c r="B82" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="C82" s="27" t="s">
+      <c r="C82" s="25" t="s">
         <v>416</v>
       </c>
       <c r="D82" s="5" t="s">
@@ -11329,7 +11327,7 @@
       <c r="B83" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C83" s="27" t="s">
+      <c r="C83" s="25" t="s">
         <v>419</v>
       </c>
       <c r="D83" s="5" t="s">
@@ -11380,7 +11378,7 @@
       <c r="B84" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C84" s="27" t="s">
+      <c r="C84" s="25" t="s">
         <v>423</v>
       </c>
       <c r="D84" s="3" t="s">
@@ -11431,7 +11429,7 @@
       <c r="B85" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C85" s="27" t="s">
+      <c r="C85" s="25" t="s">
         <v>426</v>
       </c>
       <c r="D85" s="3" t="s">
@@ -11492,7 +11490,7 @@
       <c r="B86" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C86" s="27" t="s">
+      <c r="C86" s="25" t="s">
         <v>433</v>
       </c>
       <c r="D86" s="5" t="s">
@@ -11524,7 +11522,7 @@
       </c>
       <c r="M86" s="5"/>
       <c r="N86" s="19"/>
-      <c r="O86" s="30">
+      <c r="O86" s="28">
         <v>0</v>
       </c>
       <c r="P86" s="19"/>
@@ -11547,7 +11545,7 @@
       <c r="B87" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C87" s="27" t="s">
+      <c r="C87" s="25" t="s">
         <v>437</v>
       </c>
       <c r="D87" s="3" t="s">
@@ -11579,7 +11577,7 @@
       </c>
       <c r="M87" s="3"/>
       <c r="N87" s="18"/>
-      <c r="O87" s="30">
+      <c r="O87" s="28">
         <v>0</v>
       </c>
       <c r="P87" s="18"/>
@@ -11602,7 +11600,7 @@
       <c r="B88" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C88" s="27" t="s">
+      <c r="C88" s="25" t="s">
         <v>441</v>
       </c>
       <c r="D88" s="5" t="s">
@@ -11657,7 +11655,7 @@
       <c r="B89" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C89" s="27" t="s">
+      <c r="C89" s="25" t="s">
         <v>446</v>
       </c>
       <c r="D89" s="5" t="s">
@@ -11710,7 +11708,7 @@
       <c r="B90" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C90" s="27" t="s">
+      <c r="C90" s="25" t="s">
         <v>451</v>
       </c>
       <c r="D90" s="5" t="s">
@@ -11765,7 +11763,7 @@
       <c r="B91" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C91" s="27" t="s">
+      <c r="C91" s="25" t="s">
         <v>456</v>
       </c>
       <c r="D91" s="5" t="s">
@@ -11912,39 +11910,39 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:V999"/>
+  <dimension ref="A1:U999"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="37" customWidth="1"/>
-    <col min="2" max="2" width="37" style="25" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" style="25" customWidth="1"/>
-    <col min="4" max="4" width="37" style="25" customWidth="1"/>
-    <col min="5" max="5" width="20.33203125" style="25" customWidth="1"/>
-    <col min="6" max="6" width="26.1640625" style="25" customWidth="1"/>
-    <col min="7" max="7" width="18.6640625" style="25" customWidth="1"/>
-    <col min="8" max="8" width="29" style="25" customWidth="1"/>
-    <col min="9" max="9" width="28.83203125" style="25" customWidth="1"/>
+    <col min="2" max="2" width="37" style="23" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" style="23" customWidth="1"/>
+    <col min="4" max="4" width="37" style="23" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" style="23" customWidth="1"/>
+    <col min="6" max="6" width="26.1640625" style="23" customWidth="1"/>
+    <col min="7" max="7" width="18.6640625" style="23" customWidth="1"/>
+    <col min="8" max="8" width="29" style="23" customWidth="1"/>
+    <col min="9" max="9" width="28.83203125" style="23" customWidth="1"/>
     <col min="10" max="10" width="48.1640625" customWidth="1"/>
     <col min="11" max="11" width="21.6640625" customWidth="1"/>
     <col min="12" max="12" width="20.5" customWidth="1"/>
     <col min="13" max="13" width="17" customWidth="1"/>
-    <col min="15" max="15" width="29.1640625" style="25" customWidth="1"/>
-    <col min="17" max="17" width="39.1640625" style="25" customWidth="1"/>
-    <col min="18" max="18" width="21.6640625" style="25" customWidth="1"/>
-    <col min="19" max="19" width="33.33203125" style="25" customWidth="1"/>
+    <col min="15" max="15" width="29.1640625" style="23" customWidth="1"/>
+    <col min="17" max="17" width="39.1640625" style="23" customWidth="1"/>
+    <col min="18" max="18" width="21.6640625" style="23" customWidth="1"/>
+    <col min="19" max="19" width="33.33203125" style="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="49.5" customHeight="1">
+    <row r="1" spans="1:21" ht="49.5" customHeight="1">
       <c r="A1" s="14" t="s">
         <v>460</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1149</v>
       </c>
-      <c r="C1" s="33" t="s">
+      <c r="C1" s="31" t="s">
         <v>1159</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="24" t="s">
         <v>1158</v>
       </c>
       <c r="E1" s="15" t="s">
@@ -11953,31 +11951,31 @@
       <c r="F1" s="16" t="s">
         <v>1161</v>
       </c>
-      <c r="G1" s="26" t="s">
+      <c r="G1" s="24" t="s">
         <v>1154</v>
       </c>
-      <c r="H1" s="34" t="s">
+      <c r="H1" s="32" t="s">
         <v>1162</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="32" t="s">
         <v>1163</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="32" t="s">
         <v>1164</v>
       </c>
-      <c r="K1" s="26" t="s">
+      <c r="K1" s="24" t="s">
         <v>1165</v>
       </c>
-      <c r="L1" s="26" t="s">
+      <c r="L1" s="24" t="s">
         <v>1166</v>
       </c>
       <c r="M1" t="s">
         <v>1167</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="32" t="s">
         <v>1168</v>
       </c>
-      <c r="O1" s="34" t="s">
+      <c r="O1" s="32" t="s">
         <v>1169</v>
       </c>
       <c r="P1" s="17" t="s">
@@ -11989,21 +11987,20 @@
       <c r="R1" t="s">
         <v>1170</v>
       </c>
-      <c r="S1" s="26" t="s">
+      <c r="S1" s="24" t="s">
         <v>1173</v>
       </c>
       <c r="T1" s="2"/>
       <c r="U1" s="2"/>
-      <c r="V1" s="2"/>
-    </row>
-    <row r="2" spans="1:22" ht="28">
+    </row>
+    <row r="2" spans="1:21" ht="28">
       <c r="A2" s="3" t="s">
         <v>462</v>
       </c>
       <c r="B2" s="18" t="s">
         <v>461</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="26" t="s">
         <v>463</v>
       </c>
       <c r="D2" s="19" t="s">
@@ -12039,14 +12036,14 @@
       <c r="R2" s="19"/>
       <c r="S2" s="19"/>
     </row>
-    <row r="3" spans="1:22" ht="28">
+    <row r="3" spans="1:21" ht="28">
       <c r="A3" s="5" t="s">
         <v>468</v>
       </c>
       <c r="B3" s="18" t="s">
         <v>461</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="26" t="s">
         <v>469</v>
       </c>
       <c r="D3" s="19" t="s">
@@ -12082,14 +12079,14 @@
       <c r="R3" s="19"/>
       <c r="S3" s="19"/>
     </row>
-    <row r="4" spans="1:22" ht="84">
+    <row r="4" spans="1:21" ht="84">
       <c r="A4" s="3" t="s">
         <v>470</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>461</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="26" t="s">
         <v>471</v>
       </c>
       <c r="D4" s="19" t="s">
@@ -12131,14 +12128,14 @@
       <c r="R4" s="19"/>
       <c r="S4" s="19"/>
     </row>
-    <row r="5" spans="1:22" ht="28">
+    <row r="5" spans="1:21" ht="28">
       <c r="A5" s="5" t="s">
         <v>475</v>
       </c>
       <c r="B5" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="26" t="s">
         <v>476</v>
       </c>
       <c r="D5" s="19" t="s">
@@ -12168,14 +12165,14 @@
       <c r="R5" s="19"/>
       <c r="S5" s="19"/>
     </row>
-    <row r="6" spans="1:22" ht="56">
+    <row r="6" spans="1:21" ht="56">
       <c r="A6" s="5" t="s">
         <v>479</v>
       </c>
       <c r="B6" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="28" t="s">
+      <c r="C6" s="26" t="s">
         <v>480</v>
       </c>
       <c r="D6" s="19" t="s">
@@ -12203,14 +12200,14 @@
       <c r="R6" s="19"/>
       <c r="S6" s="19"/>
     </row>
-    <row r="7" spans="1:22" ht="168">
+    <row r="7" spans="1:21" ht="168">
       <c r="A7" s="5" t="s">
         <v>484</v>
       </c>
       <c r="B7" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="28" t="s">
+      <c r="C7" s="26" t="s">
         <v>485</v>
       </c>
       <c r="D7" s="19" t="s">
@@ -12248,20 +12245,20 @@
       </c>
       <c r="S7" s="19"/>
     </row>
-    <row r="8" spans="1:22" ht="224">
+    <row r="8" spans="1:21" ht="224">
       <c r="A8" s="3" t="s">
         <v>487</v>
       </c>
       <c r="B8" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="26" t="s">
         <v>488</v>
       </c>
       <c r="D8" s="19" t="s">
         <v>489</v>
       </c>
-      <c r="E8" s="32" t="s">
+      <c r="E8" s="30" t="s">
         <v>490</v>
       </c>
       <c r="F8" s="18" t="s">
@@ -12297,14 +12294,14 @@
       <c r="R8" s="18"/>
       <c r="S8" s="18"/>
     </row>
-    <row r="9" spans="1:22" ht="70">
+    <row r="9" spans="1:21" ht="70">
       <c r="A9" s="5" t="s">
         <v>494</v>
       </c>
       <c r="B9" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="26" t="s">
         <v>495</v>
       </c>
       <c r="D9" s="19" t="s">
@@ -12332,14 +12329,14 @@
       <c r="R9" s="19"/>
       <c r="S9" s="19"/>
     </row>
-    <row r="10" spans="1:22" ht="56">
+    <row r="10" spans="1:21" ht="56">
       <c r="A10" s="5" t="s">
         <v>498</v>
       </c>
       <c r="B10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="C10" s="26" t="s">
         <v>499</v>
       </c>
       <c r="D10" s="19" t="s">
@@ -12373,14 +12370,14 @@
       <c r="R10" s="19"/>
       <c r="S10" s="19"/>
     </row>
-    <row r="11" spans="1:22" ht="56">
+    <row r="11" spans="1:21" ht="56">
       <c r="A11" s="5" t="s">
         <v>502</v>
       </c>
       <c r="B11" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="28" t="s">
+      <c r="C11" s="26" t="s">
         <v>503</v>
       </c>
       <c r="D11" s="19" t="s">
@@ -12412,14 +12409,14 @@
       <c r="R11" s="19"/>
       <c r="S11" s="19"/>
     </row>
-    <row r="12" spans="1:22" ht="56">
+    <row r="12" spans="1:21" ht="56">
       <c r="A12" s="5" t="s">
         <v>504</v>
       </c>
       <c r="B12" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="C12" s="28" t="s">
+      <c r="C12" s="26" t="s">
         <v>505</v>
       </c>
       <c r="D12" s="19" t="s">
@@ -12451,14 +12448,14 @@
       <c r="R12" s="19"/>
       <c r="S12" s="19"/>
     </row>
-    <row r="13" spans="1:22" ht="140">
+    <row r="13" spans="1:21" ht="140">
       <c r="A13" s="5" t="s">
         <v>508</v>
       </c>
       <c r="B13" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="C13" s="28" t="s">
+      <c r="C13" s="26" t="s">
         <v>509</v>
       </c>
       <c r="D13" s="19" t="s">
@@ -12494,14 +12491,14 @@
       <c r="R13" s="19"/>
       <c r="S13" s="19"/>
     </row>
-    <row r="14" spans="1:22" ht="28">
+    <row r="14" spans="1:21" ht="28">
       <c r="A14" s="5" t="s">
         <v>512</v>
       </c>
       <c r="B14" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="28" t="s">
+      <c r="C14" s="26" t="s">
         <v>513</v>
       </c>
       <c r="D14" s="19" t="s">
@@ -12529,14 +12526,14 @@
       <c r="R14" s="19"/>
       <c r="S14" s="19"/>
     </row>
-    <row r="15" spans="1:22" ht="126">
+    <row r="15" spans="1:21" ht="126">
       <c r="A15" s="5" t="s">
         <v>515</v>
       </c>
       <c r="B15" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="C15" s="28" t="s">
+      <c r="C15" s="26" t="s">
         <v>516</v>
       </c>
       <c r="D15" s="19" t="s">
@@ -12568,14 +12565,14 @@
       <c r="R15" s="19"/>
       <c r="S15" s="19"/>
     </row>
-    <row r="16" spans="1:22" ht="56">
+    <row r="16" spans="1:21" ht="56">
       <c r="A16" s="5" t="s">
         <v>517</v>
       </c>
       <c r="B16" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="28" t="s">
+      <c r="C16" s="26" t="s">
         <v>518</v>
       </c>
       <c r="D16" s="19" t="s">
@@ -12612,7 +12609,7 @@
       <c r="B17" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="C17" s="28" t="s">
+      <c r="C17" s="26" t="s">
         <v>520</v>
       </c>
       <c r="D17" s="19" t="s">
@@ -12649,7 +12646,7 @@
       <c r="B18" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="26" t="s">
         <v>522</v>
       </c>
       <c r="D18" s="19" t="s">
@@ -12686,7 +12683,7 @@
       <c r="B19" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="28" t="s">
+      <c r="C19" s="26" t="s">
         <v>524</v>
       </c>
       <c r="D19" s="19" t="s">
@@ -12723,7 +12720,7 @@
       <c r="B20" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="C20" s="28" t="s">
+      <c r="C20" s="26" t="s">
         <v>527</v>
       </c>
       <c r="D20" s="19" t="s">
@@ -12760,7 +12757,7 @@
       <c r="B21" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="C21" s="28" t="s">
+      <c r="C21" s="26" t="s">
         <v>529</v>
       </c>
       <c r="D21" s="19" t="s">
@@ -12811,7 +12808,7 @@
       <c r="B22" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="C22" s="28" t="s">
+      <c r="C22" s="26" t="s">
         <v>536</v>
       </c>
       <c r="D22" s="19" t="s">
@@ -12846,7 +12843,7 @@
       <c r="B23" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="26" t="s">
         <v>539</v>
       </c>
       <c r="D23" s="19" t="s">
@@ -12881,7 +12878,7 @@
       <c r="B24" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="C24" s="28" t="s">
+      <c r="C24" s="26" t="s">
         <v>541</v>
       </c>
       <c r="D24" s="19" t="s">
@@ -12926,7 +12923,7 @@
       <c r="B25" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="C25" s="28" t="s">
+      <c r="C25" s="26" t="s">
         <v>545</v>
       </c>
       <c r="D25" s="19" t="s">
@@ -12969,7 +12966,7 @@
       <c r="B26" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="C26" s="28" t="s">
+      <c r="C26" s="26" t="s">
         <v>549</v>
       </c>
       <c r="D26" s="19" t="s">
@@ -13012,7 +13009,7 @@
       <c r="B27" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="C27" s="28" t="s">
+      <c r="C27" s="26" t="s">
         <v>552</v>
       </c>
       <c r="D27" s="19" t="s">
@@ -13055,7 +13052,7 @@
       <c r="B28" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="C28" s="28" t="s">
+      <c r="C28" s="26" t="s">
         <v>556</v>
       </c>
       <c r="D28" s="19" t="s">
@@ -13098,7 +13095,7 @@
       <c r="B29" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="C29" s="28" t="s">
+      <c r="C29" s="26" t="s">
         <v>561</v>
       </c>
       <c r="D29" s="19" t="s">
@@ -13145,7 +13142,7 @@
       <c r="B30" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="C30" s="28" t="s">
+      <c r="C30" s="26" t="s">
         <v>564</v>
       </c>
       <c r="D30" s="19" t="s">
@@ -13192,7 +13189,7 @@
       <c r="B31" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="C31" s="28" t="s">
+      <c r="C31" s="26" t="s">
         <v>571</v>
       </c>
       <c r="D31" s="19" t="s">
@@ -13239,7 +13236,7 @@
       <c r="B32" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="C32" s="28" t="s">
+      <c r="C32" s="26" t="s">
         <v>576</v>
       </c>
       <c r="D32" s="19" t="s">
@@ -13286,7 +13283,7 @@
       <c r="B33" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="C33" s="28" t="s">
+      <c r="C33" s="26" t="s">
         <v>581</v>
       </c>
       <c r="D33" s="19" t="s">
@@ -13333,7 +13330,7 @@
       <c r="B34" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="C34" s="28" t="s">
+      <c r="C34" s="26" t="s">
         <v>585</v>
       </c>
       <c r="D34" s="19" t="s">
@@ -13378,7 +13375,7 @@
       <c r="B35" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="C35" s="28" t="s">
+      <c r="C35" s="26" t="s">
         <v>591</v>
       </c>
       <c r="D35" s="19" t="s">
@@ -13425,7 +13422,7 @@
       <c r="B36" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="C36" s="28" t="s">
+      <c r="C36" s="26" t="s">
         <v>598</v>
       </c>
       <c r="D36" s="19" t="s">
@@ -13470,7 +13467,7 @@
       <c r="B37" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="C37" s="28" t="s">
+      <c r="C37" s="26" t="s">
         <v>603</v>
       </c>
       <c r="D37" s="19" t="s">
@@ -13503,7 +13500,7 @@
       <c r="B38" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="C38" s="28" t="s">
+      <c r="C38" s="26" t="s">
         <v>605</v>
       </c>
       <c r="D38" s="19" t="s">
@@ -13544,7 +13541,7 @@
       <c r="B39" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="C39" s="28" t="s">
+      <c r="C39" s="26" t="s">
         <v>609</v>
       </c>
       <c r="D39" s="19" t="s">
@@ -13585,7 +13582,7 @@
       <c r="B40" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="C40" s="28" t="s">
+      <c r="C40" s="26" t="s">
         <v>614</v>
       </c>
       <c r="D40" s="19" t="s">
@@ -13634,7 +13631,7 @@
       <c r="B41" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="C41" s="28" t="s">
+      <c r="C41" s="26" t="s">
         <v>619</v>
       </c>
       <c r="D41" s="19" t="s">
@@ -13679,7 +13676,7 @@
       <c r="B42" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="C42" s="28" t="s">
+      <c r="C42" s="26" t="s">
         <v>625</v>
       </c>
       <c r="D42" s="19" t="s">
@@ -13720,7 +13717,7 @@
       <c r="B43" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="C43" s="28" t="s">
+      <c r="C43" s="26" t="s">
         <v>630</v>
       </c>
       <c r="D43" s="19" t="s">
@@ -13765,7 +13762,7 @@
       <c r="B44" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="C44" s="28" t="s">
+      <c r="C44" s="26" t="s">
         <v>633</v>
       </c>
       <c r="D44" s="19" t="s">
@@ -13812,7 +13809,7 @@
       <c r="B45" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="C45" s="28" t="s">
+      <c r="C45" s="26" t="s">
         <v>639</v>
       </c>
       <c r="D45" s="19" t="s">
@@ -13857,7 +13854,7 @@
       <c r="B46" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="C46" s="28" t="s">
+      <c r="C46" s="26" t="s">
         <v>643</v>
       </c>
       <c r="D46" s="19" t="s">
@@ -13906,7 +13903,7 @@
       <c r="B47" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="C47" s="28" t="s">
+      <c r="C47" s="26" t="s">
         <v>647</v>
       </c>
       <c r="D47" s="19" t="s">
@@ -13941,7 +13938,7 @@
       <c r="B48" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="C48" s="28" t="s">
+      <c r="C48" s="26" t="s">
         <v>649</v>
       </c>
       <c r="D48" s="19" t="s">
@@ -13974,7 +13971,7 @@
       <c r="B49" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="C49" s="28" t="s">
+      <c r="C49" s="26" t="s">
         <v>651</v>
       </c>
       <c r="D49" s="19" t="s">
@@ -14007,7 +14004,7 @@
       <c r="B50" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C50" s="28" t="s">
+      <c r="C50" s="26" t="s">
         <v>653</v>
       </c>
       <c r="D50" s="19" t="s">
@@ -14035,14 +14032,14 @@
       <c r="R50" s="19"/>
       <c r="S50" s="19"/>
     </row>
-    <row r="51" spans="1:19" ht="112">
+    <row r="51" spans="1:19" ht="84">
       <c r="A51" s="3" t="s">
         <v>654</v>
       </c>
       <c r="B51" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="C51" s="28" t="s">
+      <c r="C51" s="26" t="s">
         <v>655</v>
       </c>
       <c r="D51" s="19" t="s">
@@ -14087,7 +14084,7 @@
       <c r="B52" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="C52" s="28" t="s">
+      <c r="C52" s="26" t="s">
         <v>661</v>
       </c>
       <c r="D52" s="19" t="s">
@@ -14169,7 +14166,7 @@
       <c r="B54" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="C54" s="28" t="s">
+      <c r="C54" s="26" t="s">
         <v>667</v>
       </c>
       <c r="D54" s="19" t="s">
@@ -14218,7 +14215,7 @@
       <c r="B55" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="C55" s="28" t="s">
+      <c r="C55" s="26" t="s">
         <v>671</v>
       </c>
       <c r="D55" s="19" t="s">
@@ -14267,7 +14264,7 @@
       <c r="B56" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="C56" s="28" t="s">
+      <c r="C56" s="26" t="s">
         <v>676</v>
       </c>
       <c r="D56" s="19" t="s">
@@ -14304,7 +14301,7 @@
       <c r="B57" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="C57" s="28" t="s">
+      <c r="C57" s="26" t="s">
         <v>678</v>
       </c>
       <c r="D57" s="19" t="s">
@@ -14359,7 +14356,7 @@
       <c r="B58" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="C58" s="28" t="s">
+      <c r="C58" s="26" t="s">
         <v>683</v>
       </c>
       <c r="D58" s="19" t="s">
@@ -14396,7 +14393,7 @@
       <c r="B59" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="C59" s="28" t="s">
+      <c r="C59" s="26" t="s">
         <v>685</v>
       </c>
       <c r="D59" s="19" t="s">
@@ -14447,7 +14444,7 @@
       <c r="B60" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="C60" s="28" t="s">
+      <c r="C60" s="26" t="s">
         <v>689</v>
       </c>
       <c r="D60" s="19" t="s">
@@ -14500,7 +14497,7 @@
       <c r="B61" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="C61" s="28" t="s">
+      <c r="C61" s="26" t="s">
         <v>692</v>
       </c>
       <c r="D61" s="19" t="s">
@@ -14545,7 +14542,7 @@
       <c r="B62" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="C62" s="28" t="s">
+      <c r="C62" s="26" t="s">
         <v>695</v>
       </c>
       <c r="D62" s="19" t="s">
@@ -14588,7 +14585,7 @@
       <c r="B63" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="C63" s="28" t="s">
+      <c r="C63" s="26" t="s">
         <v>699</v>
       </c>
       <c r="D63" s="19" t="s">
@@ -14637,7 +14634,7 @@
       <c r="B64" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="C64" s="28" t="s">
+      <c r="C64" s="26" t="s">
         <v>704</v>
       </c>
       <c r="D64" s="19" t="s">
@@ -14680,7 +14677,7 @@
       <c r="B65" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="C65" s="28" t="s">
+      <c r="C65" s="26" t="s">
         <v>707</v>
       </c>
       <c r="D65" s="19" t="s">
@@ -14719,7 +14716,7 @@
       <c r="B66" s="18" t="s">
         <v>172</v>
       </c>
-      <c r="C66" s="28" t="s">
+      <c r="C66" s="26" t="s">
         <v>710</v>
       </c>
       <c r="D66" s="19" t="s">
@@ -14762,7 +14759,7 @@
       <c r="B67" s="18" t="s">
         <v>172</v>
       </c>
-      <c r="C67" s="28" t="s">
+      <c r="C67" s="26" t="s">
         <v>712</v>
       </c>
       <c r="D67" s="19" t="s">
@@ -14801,7 +14798,7 @@
       <c r="B68" s="18" t="s">
         <v>172</v>
       </c>
-      <c r="C68" s="28" t="s">
+      <c r="C68" s="26" t="s">
         <v>715</v>
       </c>
       <c r="D68" s="19" t="s">
@@ -14840,7 +14837,7 @@
       <c r="B69" s="19" t="s">
         <v>177</v>
       </c>
-      <c r="C69" s="28" t="s">
+      <c r="C69" s="26" t="s">
         <v>718</v>
       </c>
       <c r="D69" s="19" t="s">
@@ -14891,7 +14888,7 @@
       <c r="B70" s="19" t="s">
         <v>185</v>
       </c>
-      <c r="C70" s="28" t="s">
+      <c r="C70" s="26" t="s">
         <v>724</v>
       </c>
       <c r="D70" s="19" t="s">
@@ -14926,7 +14923,7 @@
       <c r="B71" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="C71" s="28" t="s">
+      <c r="C71" s="26" t="s">
         <v>726</v>
       </c>
       <c r="D71" s="19" t="s">
@@ -14961,7 +14958,7 @@
       <c r="B72" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="C72" s="28" t="s">
+      <c r="C72" s="26" t="s">
         <v>728</v>
       </c>
       <c r="D72" s="19" t="s">
@@ -15014,7 +15011,7 @@
       <c r="B73" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="C73" s="28" t="s">
+      <c r="C73" s="26" t="s">
         <v>732</v>
       </c>
       <c r="D73" s="19" t="s">
@@ -15067,7 +15064,7 @@
       <c r="B74" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="C74" s="28" t="s">
+      <c r="C74" s="26" t="s">
         <v>735</v>
       </c>
       <c r="D74" s="19" t="s">
@@ -15120,7 +15117,7 @@
       <c r="B75" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="C75" s="28" t="s">
+      <c r="C75" s="26" t="s">
         <v>738</v>
       </c>
       <c r="D75" s="19" t="s">
@@ -15173,7 +15170,7 @@
       <c r="B76" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="C76" s="28" t="s">
+      <c r="C76" s="26" t="s">
         <v>741</v>
       </c>
       <c r="D76" s="19" t="s">
@@ -15226,7 +15223,7 @@
       <c r="B77" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="C77" s="28" t="s">
+      <c r="C77" s="26" t="s">
         <v>745</v>
       </c>
       <c r="D77" s="19" t="s">
@@ -15279,7 +15276,7 @@
       <c r="B78" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="C78" s="28" t="s">
+      <c r="C78" s="26" t="s">
         <v>748</v>
       </c>
       <c r="D78" s="19" t="s">
@@ -15332,7 +15329,7 @@
       <c r="B79" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="C79" s="28" t="s">
+      <c r="C79" s="26" t="s">
         <v>751</v>
       </c>
       <c r="D79" s="19" t="s">
@@ -15385,7 +15382,7 @@
       <c r="B80" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="C80" s="28" t="s">
+      <c r="C80" s="26" t="s">
         <v>754</v>
       </c>
       <c r="D80" s="19" t="s">
@@ -15438,7 +15435,7 @@
       <c r="B81" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="C81" s="28" t="s">
+      <c r="C81" s="26" t="s">
         <v>758</v>
       </c>
       <c r="D81" s="19" t="s">
@@ -15491,7 +15488,7 @@
       <c r="B82" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="C82" s="28" t="s">
+      <c r="C82" s="26" t="s">
         <v>761</v>
       </c>
       <c r="D82" s="19" t="s">
@@ -15544,7 +15541,7 @@
       <c r="B83" s="18" t="s">
         <v>199</v>
       </c>
-      <c r="C83" s="28" t="s">
+      <c r="C83" s="26" t="s">
         <v>764</v>
       </c>
       <c r="D83" s="19" t="s">
@@ -15597,7 +15594,7 @@
       <c r="B84" s="18" t="s">
         <v>199</v>
       </c>
-      <c r="C84" s="28" t="s">
+      <c r="C84" s="26" t="s">
         <v>767</v>
       </c>
       <c r="D84" s="19" t="s">
@@ -15650,7 +15647,7 @@
       <c r="B85" s="18" t="s">
         <v>199</v>
       </c>
-      <c r="C85" s="28" t="s">
+      <c r="C85" s="26" t="s">
         <v>771</v>
       </c>
       <c r="D85" s="19" t="s">
@@ -15701,7 +15698,7 @@
       <c r="B86" s="18" t="s">
         <v>199</v>
       </c>
-      <c r="C86" s="28" t="s">
+      <c r="C86" s="26" t="s">
         <v>776</v>
       </c>
       <c r="D86" s="19" t="s">
@@ -15754,7 +15751,7 @@
       <c r="B87" s="18" t="s">
         <v>199</v>
       </c>
-      <c r="C87" s="28" t="s">
+      <c r="C87" s="26" t="s">
         <v>783</v>
       </c>
       <c r="D87" s="19" t="s">
@@ -15807,7 +15804,7 @@
       <c r="B88" s="18" t="s">
         <v>199</v>
       </c>
-      <c r="C88" s="28" t="s">
+      <c r="C88" s="26" t="s">
         <v>789</v>
       </c>
       <c r="D88" s="19" t="s">
@@ -15858,7 +15855,7 @@
       <c r="B89" s="18" t="s">
         <v>199</v>
       </c>
-      <c r="C89" s="28" t="s">
+      <c r="C89" s="26" t="s">
         <v>795</v>
       </c>
       <c r="D89" s="19" t="s">
@@ -15910,10 +15907,10 @@
       <c r="A90" s="11" t="s">
         <v>800</v>
       </c>
-      <c r="B90" s="24" t="s">
+      <c r="B90" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="C90" s="28" t="s">
+      <c r="C90" s="26" t="s">
         <v>801</v>
       </c>
       <c r="D90" s="19" t="s">
@@ -15956,7 +15953,7 @@
       <c r="B91" s="19" t="s">
         <v>212</v>
       </c>
-      <c r="C91" s="28" t="s">
+      <c r="C91" s="26" t="s">
         <v>803</v>
       </c>
       <c r="D91" s="19" t="s">
@@ -15995,7 +15992,7 @@
       <c r="B92" s="19" t="s">
         <v>212</v>
       </c>
-      <c r="C92" s="28" t="s">
+      <c r="C92" s="26" t="s">
         <v>805</v>
       </c>
       <c r="D92" s="19" t="s">
@@ -16034,7 +16031,7 @@
       <c r="B93" s="19" t="s">
         <v>212</v>
       </c>
-      <c r="C93" s="28" t="s">
+      <c r="C93" s="26" t="s">
         <v>807</v>
       </c>
       <c r="D93" s="19" t="s">
@@ -16071,7 +16068,7 @@
       <c r="B94" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="C94" s="28" t="s">
+      <c r="C94" s="26" t="s">
         <v>809</v>
       </c>
       <c r="D94" s="19" t="s">
@@ -16114,7 +16111,7 @@
       <c r="B95" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="C95" s="28" t="s">
+      <c r="C95" s="26" t="s">
         <v>812</v>
       </c>
       <c r="D95" s="19" t="s">
@@ -16153,7 +16150,7 @@
       <c r="B96" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="C96" s="28" t="s">
+      <c r="C96" s="26" t="s">
         <v>816</v>
       </c>
       <c r="D96" s="19" t="s">
@@ -16204,7 +16201,7 @@
       <c r="B97" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="C97" s="28" t="s">
+      <c r="C97" s="26" t="s">
         <v>819</v>
       </c>
       <c r="D97" s="19" t="s">
@@ -16255,7 +16252,7 @@
       <c r="B98" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="C98" s="28" t="s">
+      <c r="C98" s="26" t="s">
         <v>824</v>
       </c>
       <c r="D98" s="19" t="s">
@@ -16300,7 +16297,7 @@
       <c r="B99" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="C99" s="28" t="s">
+      <c r="C99" s="26" t="s">
         <v>830</v>
       </c>
       <c r="D99" s="19" t="s">
@@ -16343,7 +16340,7 @@
       <c r="B100" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="C100" s="28" t="s">
+      <c r="C100" s="26" t="s">
         <v>835</v>
       </c>
       <c r="D100" s="19" t="s">
@@ -16386,7 +16383,7 @@
       <c r="B101" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="C101" s="28" t="s">
+      <c r="C101" s="26" t="s">
         <v>840</v>
       </c>
       <c r="D101" s="19" t="s">
@@ -16429,7 +16426,7 @@
       <c r="B102" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="C102" s="28" t="s">
+      <c r="C102" s="26" t="s">
         <v>844</v>
       </c>
       <c r="D102" s="19" t="s">
@@ -16480,7 +16477,7 @@
       <c r="B103" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="C103" s="28" t="s">
+      <c r="C103" s="26" t="s">
         <v>849</v>
       </c>
       <c r="D103" s="19" t="s">
@@ -16519,7 +16516,7 @@
       <c r="B104" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="C104" s="28" t="s">
+      <c r="C104" s="26" t="s">
         <v>853</v>
       </c>
       <c r="D104" s="19" t="s">
@@ -16558,7 +16555,7 @@
       <c r="B105" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="C105" s="28" t="s">
+      <c r="C105" s="26" t="s">
         <v>856</v>
       </c>
       <c r="D105" s="19" t="s">
@@ -16597,7 +16594,7 @@
       <c r="B106" s="19" t="s">
         <v>236</v>
       </c>
-      <c r="C106" s="28" t="s">
+      <c r="C106" s="26" t="s">
         <v>859</v>
       </c>
       <c r="D106" s="19" t="s">
@@ -16625,14 +16622,14 @@
       <c r="R106" s="19"/>
       <c r="S106" s="19"/>
     </row>
-    <row r="107" spans="1:19" ht="112">
+    <row r="107" spans="1:19" ht="84">
       <c r="A107" s="5" t="s">
         <v>239</v>
       </c>
       <c r="B107" s="19" t="s">
         <v>239</v>
       </c>
-      <c r="C107" s="28" t="s">
+      <c r="C107" s="26" t="s">
         <v>860</v>
       </c>
       <c r="D107" s="19" t="s">
@@ -16689,7 +16686,7 @@
       <c r="B108" s="19" t="s">
         <v>250</v>
       </c>
-      <c r="C108" s="28" t="s">
+      <c r="C108" s="26" t="s">
         <v>864</v>
       </c>
       <c r="D108" s="19" t="s">
@@ -16734,7 +16731,7 @@
       <c r="B109" s="19" t="s">
         <v>250</v>
       </c>
-      <c r="C109" s="28" t="s">
+      <c r="C109" s="26" t="s">
         <v>866</v>
       </c>
       <c r="D109" s="19" t="s">
@@ -16779,7 +16776,7 @@
       <c r="B110" s="19" t="s">
         <v>250</v>
       </c>
-      <c r="C110" s="28" t="s">
+      <c r="C110" s="26" t="s">
         <v>871</v>
       </c>
       <c r="D110" s="19" t="s">
@@ -16822,7 +16819,7 @@
       <c r="B111" s="19" t="s">
         <v>250</v>
       </c>
-      <c r="C111" s="28" t="s">
+      <c r="C111" s="26" t="s">
         <v>873</v>
       </c>
       <c r="D111" s="19" t="s">
@@ -16867,7 +16864,7 @@
       <c r="B112" s="19" t="s">
         <v>255</v>
       </c>
-      <c r="C112" s="28" t="s">
+      <c r="C112" s="26" t="s">
         <v>877</v>
       </c>
       <c r="D112" s="19" t="s">
@@ -16906,7 +16903,7 @@
       <c r="B113" s="19" t="s">
         <v>258</v>
       </c>
-      <c r="C113" s="28" t="s">
+      <c r="C113" s="26" t="s">
         <v>879</v>
       </c>
       <c r="D113" s="19" t="s">
@@ -16945,7 +16942,7 @@
       <c r="B114" s="19" t="s">
         <v>258</v>
       </c>
-      <c r="C114" s="28" t="s">
+      <c r="C114" s="26" t="s">
         <v>881</v>
       </c>
       <c r="D114" s="19" t="s">
@@ -16984,7 +16981,7 @@
       <c r="B115" s="19" t="s">
         <v>258</v>
       </c>
-      <c r="C115" s="28" t="s">
+      <c r="C115" s="26" t="s">
         <v>883</v>
       </c>
       <c r="D115" s="19" t="s">
@@ -17023,7 +17020,7 @@
       <c r="B116" s="19" t="s">
         <v>261</v>
       </c>
-      <c r="C116" s="28" t="s">
+      <c r="C116" s="26" t="s">
         <v>885</v>
       </c>
       <c r="D116" s="19" t="s">
@@ -17076,7 +17073,7 @@
       <c r="B117" s="19" t="s">
         <v>268</v>
       </c>
-      <c r="C117" s="28" t="s">
+      <c r="C117" s="26" t="s">
         <v>889</v>
       </c>
       <c r="D117" s="19" t="s">
@@ -17115,7 +17112,7 @@
       <c r="B118" s="19" t="s">
         <v>268</v>
       </c>
-      <c r="C118" s="28" t="s">
+      <c r="C118" s="26" t="s">
         <v>891</v>
       </c>
       <c r="D118" s="19" t="s">
@@ -17154,7 +17151,7 @@
       <c r="B119" s="19" t="s">
         <v>273</v>
       </c>
-      <c r="C119" s="28" t="s">
+      <c r="C119" s="26" t="s">
         <v>895</v>
       </c>
       <c r="D119" s="19" t="s">
@@ -17193,7 +17190,7 @@
       <c r="B120" s="19" t="s">
         <v>277</v>
       </c>
-      <c r="C120" s="28" t="s">
+      <c r="C120" s="26" t="s">
         <v>897</v>
       </c>
       <c r="D120" s="19" t="s">
@@ -17236,7 +17233,7 @@
       <c r="B121" s="19" t="s">
         <v>281</v>
       </c>
-      <c r="C121" s="28" t="s">
+      <c r="C121" s="26" t="s">
         <v>899</v>
       </c>
       <c r="D121" s="19" t="s">
@@ -17287,7 +17284,7 @@
       <c r="B122" s="19" t="s">
         <v>290</v>
       </c>
-      <c r="C122" s="28" t="s">
+      <c r="C122" s="26" t="s">
         <v>902</v>
       </c>
       <c r="D122" s="19" t="s">
@@ -17326,7 +17323,7 @@
       <c r="B123" s="19" t="s">
         <v>293</v>
       </c>
-      <c r="C123" s="28" t="s">
+      <c r="C123" s="26" t="s">
         <v>905</v>
       </c>
       <c r="D123" s="19" t="s">
@@ -17363,7 +17360,7 @@
       <c r="B124" s="19" t="s">
         <v>293</v>
       </c>
-      <c r="C124" s="28" t="s">
+      <c r="C124" s="26" t="s">
         <v>907</v>
       </c>
       <c r="D124" s="19" t="s">
@@ -17400,7 +17397,7 @@
       <c r="B125" s="19" t="s">
         <v>296</v>
       </c>
-      <c r="C125" s="28" t="s">
+      <c r="C125" s="26" t="s">
         <v>911</v>
       </c>
       <c r="D125" s="19" t="s">
@@ -17435,7 +17432,7 @@
       <c r="B126" s="19" t="s">
         <v>298</v>
       </c>
-      <c r="C126" s="28" t="s">
+      <c r="C126" s="26" t="s">
         <v>913</v>
       </c>
       <c r="D126" s="19" t="s">
@@ -17484,7 +17481,7 @@
       <c r="B127" s="19" t="s">
         <v>305</v>
       </c>
-      <c r="C127" s="28" t="s">
+      <c r="C127" s="26" t="s">
         <v>917</v>
       </c>
       <c r="D127" s="19" t="s">
@@ -17523,7 +17520,7 @@
       <c r="B128" s="19" t="s">
         <v>305</v>
       </c>
-      <c r="C128" s="28" t="s">
+      <c r="C128" s="26" t="s">
         <v>920</v>
       </c>
       <c r="D128" s="19" t="s">
@@ -17564,7 +17561,7 @@
       <c r="B129" s="19" t="s">
         <v>309</v>
       </c>
-      <c r="C129" s="28" t="s">
+      <c r="C129" s="26" t="s">
         <v>922</v>
       </c>
       <c r="D129" s="19" t="s">
@@ -17601,7 +17598,7 @@
       <c r="B130" s="18" t="s">
         <v>313</v>
       </c>
-      <c r="C130" s="28" t="s">
+      <c r="C130" s="26" t="s">
         <v>924</v>
       </c>
       <c r="D130" s="19" t="s">
@@ -17642,7 +17639,7 @@
       <c r="B131" s="18" t="s">
         <v>316</v>
       </c>
-      <c r="C131" s="28" t="s">
+      <c r="C131" s="26" t="s">
         <v>928</v>
       </c>
       <c r="D131" s="19" t="s">
@@ -17677,7 +17674,7 @@
       <c r="B132" s="18" t="s">
         <v>319</v>
       </c>
-      <c r="C132" s="28" t="s">
+      <c r="C132" s="26" t="s">
         <v>930</v>
       </c>
       <c r="D132" s="19" t="s">
@@ -17720,7 +17717,7 @@
       <c r="B133" s="18" t="s">
         <v>319</v>
       </c>
-      <c r="C133" s="28" t="s">
+      <c r="C133" s="26" t="s">
         <v>932</v>
       </c>
       <c r="D133" s="19" t="s">
@@ -17761,7 +17758,7 @@
       <c r="B134" s="18" t="s">
         <v>319</v>
       </c>
-      <c r="C134" s="28" t="s">
+      <c r="C134" s="26" t="s">
         <v>934</v>
       </c>
       <c r="D134" s="19" t="s">
@@ -17806,7 +17803,7 @@
       <c r="B135" s="18" t="s">
         <v>319</v>
       </c>
-      <c r="C135" s="28" t="s">
+      <c r="C135" s="26" t="s">
         <v>940</v>
       </c>
       <c r="D135" s="19" t="s">
@@ -17855,7 +17852,7 @@
       <c r="B136" s="18" t="s">
         <v>319</v>
       </c>
-      <c r="C136" s="28" t="s">
+      <c r="C136" s="26" t="s">
         <v>945</v>
       </c>
       <c r="D136" s="19" t="s">
@@ -17904,7 +17901,7 @@
       <c r="B137" s="19" t="s">
         <v>325</v>
       </c>
-      <c r="C137" s="28" t="s">
+      <c r="C137" s="26" t="s">
         <v>949</v>
       </c>
       <c r="D137" s="19" t="s">
@@ -17947,7 +17944,7 @@
       <c r="B138" s="19" t="s">
         <v>325</v>
       </c>
-      <c r="C138" s="28" t="s">
+      <c r="C138" s="26" t="s">
         <v>951</v>
       </c>
       <c r="D138" s="19" t="s">
@@ -17990,7 +17987,7 @@
       <c r="B139" s="19" t="s">
         <v>325</v>
       </c>
-      <c r="C139" s="28" t="s">
+      <c r="C139" s="26" t="s">
         <v>954</v>
       </c>
       <c r="D139" s="19" t="s">
@@ -18033,7 +18030,7 @@
       <c r="B140" s="18" t="s">
         <v>329</v>
       </c>
-      <c r="C140" s="28" t="s">
+      <c r="C140" s="26" t="s">
         <v>958</v>
       </c>
       <c r="D140" s="19" t="s">
@@ -18068,7 +18065,7 @@
       <c r="B141" s="19" t="s">
         <v>332</v>
       </c>
-      <c r="C141" s="28" t="s">
+      <c r="C141" s="26" t="s">
         <v>960</v>
       </c>
       <c r="D141" s="19" t="s">
@@ -18105,7 +18102,7 @@
       <c r="B142" s="19" t="s">
         <v>332</v>
       </c>
-      <c r="C142" s="28" t="s">
+      <c r="C142" s="26" t="s">
         <v>962</v>
       </c>
       <c r="D142" s="19" t="s">
@@ -18144,7 +18141,7 @@
       <c r="B143" s="19" t="s">
         <v>335</v>
       </c>
-      <c r="C143" s="28" t="s">
+      <c r="C143" s="26" t="s">
         <v>966</v>
       </c>
       <c r="D143" s="19" t="s">
@@ -18179,7 +18176,7 @@
       <c r="B144" s="19" t="s">
         <v>338</v>
       </c>
-      <c r="C144" s="28" t="s">
+      <c r="C144" s="26" t="s">
         <v>968</v>
       </c>
       <c r="D144" s="19" t="s">
@@ -18218,7 +18215,7 @@
       <c r="B145" s="19" t="s">
         <v>338</v>
       </c>
-      <c r="C145" s="28" t="s">
+      <c r="C145" s="26" t="s">
         <v>971</v>
       </c>
       <c r="D145" s="19" t="s">
@@ -18257,7 +18254,7 @@
       <c r="B146" s="19" t="s">
         <v>338</v>
       </c>
-      <c r="C146" s="28" t="s">
+      <c r="C146" s="26" t="s">
         <v>972</v>
       </c>
       <c r="D146" s="19" t="s">
@@ -18296,7 +18293,7 @@
       <c r="B147" s="19" t="s">
         <v>338</v>
       </c>
-      <c r="C147" s="28" t="s">
+      <c r="C147" s="26" t="s">
         <v>974</v>
       </c>
       <c r="D147" s="19" t="s">
@@ -18339,7 +18336,7 @@
       <c r="B148" s="19" t="s">
         <v>342</v>
       </c>
-      <c r="C148" s="28" t="s">
+      <c r="C148" s="26" t="s">
         <v>976</v>
       </c>
       <c r="D148" s="19" t="s">
@@ -18396,7 +18393,7 @@
       <c r="B149" s="19" t="s">
         <v>350</v>
       </c>
-      <c r="C149" s="28" t="s">
+      <c r="C149" s="26" t="s">
         <v>978</v>
       </c>
       <c r="D149" s="19" t="s">
@@ -18439,7 +18436,7 @@
       <c r="B150" s="19" t="s">
         <v>350</v>
       </c>
-      <c r="C150" s="28" t="s">
+      <c r="C150" s="26" t="s">
         <v>981</v>
       </c>
       <c r="D150" s="19" t="s">
@@ -18478,7 +18475,7 @@
       <c r="B151" s="19" t="s">
         <v>350</v>
       </c>
-      <c r="C151" s="28" t="s">
+      <c r="C151" s="26" t="s">
         <v>985</v>
       </c>
       <c r="D151" s="19" t="s">
@@ -18515,7 +18512,7 @@
       <c r="B152" s="19" t="s">
         <v>354</v>
       </c>
-      <c r="C152" s="28" t="s">
+      <c r="C152" s="26" t="s">
         <v>988</v>
       </c>
       <c r="D152" s="19" t="s">
@@ -18556,7 +18553,7 @@
       <c r="B153" s="19" t="s">
         <v>354</v>
       </c>
-      <c r="C153" s="28" t="s">
+      <c r="C153" s="26" t="s">
         <v>990</v>
       </c>
       <c r="D153" s="19" t="s">
@@ -18599,7 +18596,7 @@
       <c r="B154" s="19" t="s">
         <v>354</v>
       </c>
-      <c r="C154" s="28" t="s">
+      <c r="C154" s="26" t="s">
         <v>994</v>
       </c>
       <c r="D154" s="19" t="s">
@@ -18636,7 +18633,7 @@
       <c r="B155" s="19" t="s">
         <v>358</v>
       </c>
-      <c r="C155" s="28" t="s">
+      <c r="C155" s="26" t="s">
         <v>996</v>
       </c>
       <c r="D155" s="19" t="s">
@@ -18673,7 +18670,7 @@
       <c r="B156" s="19" t="s">
         <v>362</v>
       </c>
-      <c r="C156" s="28" t="s">
+      <c r="C156" s="26" t="s">
         <v>999</v>
       </c>
       <c r="D156" s="19" t="s">
@@ -18712,7 +18709,7 @@
       <c r="B157" s="19" t="s">
         <v>366</v>
       </c>
-      <c r="C157" s="28" t="s">
+      <c r="C157" s="26" t="s">
         <v>1001</v>
       </c>
       <c r="D157" s="19" t="s">
@@ -18757,7 +18754,7 @@
       <c r="B158" s="19" t="s">
         <v>366</v>
       </c>
-      <c r="C158" s="28" t="s">
+      <c r="C158" s="26" t="s">
         <v>1003</v>
       </c>
       <c r="D158" s="19" t="s">
@@ -18802,7 +18799,7 @@
       <c r="B159" s="19" t="s">
         <v>366</v>
       </c>
-      <c r="C159" s="28" t="s">
+      <c r="C159" s="26" t="s">
         <v>1008</v>
       </c>
       <c r="D159" s="19" t="s">
@@ -18845,7 +18842,7 @@
       <c r="B160" s="19" t="s">
         <v>370</v>
       </c>
-      <c r="C160" s="28" t="s">
+      <c r="C160" s="26" t="s">
         <v>1013</v>
       </c>
       <c r="D160" s="19" t="s">
@@ -18884,7 +18881,7 @@
       <c r="B161" s="19" t="s">
         <v>374</v>
       </c>
-      <c r="C161" s="28" t="s">
+      <c r="C161" s="26" t="s">
         <v>1015</v>
       </c>
       <c r="D161" s="19" t="s">
@@ -18919,7 +18916,7 @@
       <c r="B162" s="19" t="s">
         <v>376</v>
       </c>
-      <c r="C162" s="28" t="s">
+      <c r="C162" s="26" t="s">
         <v>1017</v>
       </c>
       <c r="D162" s="19" t="s">
@@ -18960,7 +18957,7 @@
       <c r="B163" s="19" t="s">
         <v>376</v>
       </c>
-      <c r="C163" s="28" t="s">
+      <c r="C163" s="26" t="s">
         <v>1020</v>
       </c>
       <c r="D163" s="19" t="s">
@@ -18999,7 +18996,7 @@
       <c r="B164" s="19" t="s">
         <v>380</v>
       </c>
-      <c r="C164" s="28" t="s">
+      <c r="C164" s="26" t="s">
         <v>1024</v>
       </c>
       <c r="D164" s="19" t="s">
@@ -19040,7 +19037,7 @@
       <c r="B165" s="19" t="s">
         <v>384</v>
       </c>
-      <c r="C165" s="28" t="s">
+      <c r="C165" s="26" t="s">
         <v>385</v>
       </c>
       <c r="D165" s="19" t="s">
@@ -19085,7 +19082,7 @@
       <c r="B166" s="19" t="s">
         <v>387</v>
       </c>
-      <c r="C166" s="28" t="s">
+      <c r="C166" s="26" t="s">
         <v>1028</v>
       </c>
       <c r="D166" s="19" t="s">
@@ -19124,7 +19121,7 @@
       <c r="B167" s="19" t="s">
         <v>387</v>
       </c>
-      <c r="C167" s="28" t="s">
+      <c r="C167" s="26" t="s">
         <v>1030</v>
       </c>
       <c r="D167" s="19" t="s">
@@ -19163,7 +19160,7 @@
       <c r="B168" s="19" t="s">
         <v>387</v>
       </c>
-      <c r="C168" s="28" t="s">
+      <c r="C168" s="26" t="s">
         <v>1032</v>
       </c>
       <c r="D168" s="19" t="s">
@@ -19202,7 +19199,7 @@
       <c r="B169" s="19" t="s">
         <v>387</v>
       </c>
-      <c r="C169" s="28" t="s">
+      <c r="C169" s="26" t="s">
         <v>1034</v>
       </c>
       <c r="D169" s="19" t="s">
@@ -19239,7 +19236,7 @@
       <c r="B170" s="19" t="s">
         <v>390</v>
       </c>
-      <c r="C170" s="28" t="s">
+      <c r="C170" s="26" t="s">
         <v>1037</v>
       </c>
       <c r="D170" s="19" t="s">
@@ -19286,7 +19283,7 @@
       <c r="B171" s="19" t="s">
         <v>395</v>
       </c>
-      <c r="C171" s="28" t="s">
+      <c r="C171" s="26" t="s">
         <v>1040</v>
       </c>
       <c r="D171" s="19" t="s">
@@ -19340,10 +19337,10 @@
       <c r="A172" s="3" t="s">
         <v>1043</v>
       </c>
-      <c r="B172" s="24" t="s">
+      <c r="B172" s="22" t="s">
         <v>401</v>
       </c>
-      <c r="C172" s="28" t="s">
+      <c r="C172" s="26" t="s">
         <v>1044</v>
       </c>
       <c r="D172" s="19" t="s">
@@ -19382,7 +19379,7 @@
       <c r="B173" s="18" t="s">
         <v>404</v>
       </c>
-      <c r="C173" s="28" t="s">
+      <c r="C173" s="26" t="s">
         <v>1046</v>
       </c>
       <c r="D173" s="19" t="s">
@@ -19435,7 +19432,7 @@
       <c r="B174" s="18" t="s">
         <v>412</v>
       </c>
-      <c r="C174" s="28" t="s">
+      <c r="C174" s="26" t="s">
         <v>1048</v>
       </c>
       <c r="D174" s="19" t="s">
@@ -19474,7 +19471,7 @@
       <c r="B175" s="18" t="s">
         <v>412</v>
       </c>
-      <c r="C175" s="28" t="s">
+      <c r="C175" s="26" t="s">
         <v>1050</v>
       </c>
       <c r="D175" s="19" t="s">
@@ -19511,7 +19508,7 @@
       <c r="B176" s="18" t="s">
         <v>412</v>
       </c>
-      <c r="C176" s="28" t="s">
+      <c r="C176" s="26" t="s">
         <v>1053</v>
       </c>
       <c r="D176" s="19" t="s">
@@ -19554,7 +19551,7 @@
       <c r="B177" s="18" t="s">
         <v>412</v>
       </c>
-      <c r="C177" s="28" t="s">
+      <c r="C177" s="26" t="s">
         <v>1056</v>
       </c>
       <c r="D177" s="19" t="s">
@@ -19593,7 +19590,7 @@
       <c r="B178" s="19" t="s">
         <v>415</v>
       </c>
-      <c r="C178" s="28" t="s">
+      <c r="C178" s="26" t="s">
         <v>1059</v>
       </c>
       <c r="D178" s="19" t="s">
@@ -19632,7 +19629,7 @@
       <c r="B179" s="19" t="s">
         <v>418</v>
       </c>
-      <c r="C179" s="28" t="s">
+      <c r="C179" s="26" t="s">
         <v>1061</v>
       </c>
       <c r="D179" s="19" t="s">
@@ -19667,7 +19664,7 @@
       <c r="B180" s="18" t="s">
         <v>422</v>
       </c>
-      <c r="C180" s="28" t="s">
+      <c r="C180" s="26" t="s">
         <v>1063</v>
       </c>
       <c r="D180" s="19" t="s">
@@ -19704,7 +19701,7 @@
       <c r="B181" s="18" t="s">
         <v>422</v>
       </c>
-      <c r="C181" s="28" t="s">
+      <c r="C181" s="26" t="s">
         <v>1065</v>
       </c>
       <c r="D181" s="19" t="s">
@@ -19741,7 +19738,7 @@
       <c r="B182" s="18" t="s">
         <v>425</v>
       </c>
-      <c r="C182" s="28" t="s">
+      <c r="C182" s="26" t="s">
         <v>1067</v>
       </c>
       <c r="D182" s="19" t="s">
@@ -19794,7 +19791,7 @@
       <c r="B183" s="18" t="s">
         <v>425</v>
       </c>
-      <c r="C183" s="28" t="s">
+      <c r="C183" s="26" t="s">
         <v>1071</v>
       </c>
       <c r="D183" s="19" t="s">
@@ -19845,7 +19842,7 @@
       <c r="B184" s="18" t="s">
         <v>425</v>
       </c>
-      <c r="C184" s="28" t="s">
+      <c r="C184" s="26" t="s">
         <v>1075</v>
       </c>
       <c r="D184" s="19" t="s">
@@ -19896,7 +19893,7 @@
       <c r="B185" s="18" t="s">
         <v>425</v>
       </c>
-      <c r="C185" s="28" t="s">
+      <c r="C185" s="26" t="s">
         <v>1079</v>
       </c>
       <c r="D185" s="19" t="s">
@@ -19949,7 +19946,7 @@
       <c r="B186" s="18" t="s">
         <v>425</v>
       </c>
-      <c r="C186" s="28" t="s">
+      <c r="C186" s="26" t="s">
         <v>1085</v>
       </c>
       <c r="D186" s="19" t="s">
@@ -19988,7 +19985,7 @@
       <c r="B187" s="18" t="s">
         <v>425</v>
       </c>
-      <c r="C187" s="28" t="s">
+      <c r="C187" s="26" t="s">
         <v>1088</v>
       </c>
       <c r="D187" s="19" t="s">
@@ -20037,7 +20034,7 @@
       <c r="B188" s="18" t="s">
         <v>432</v>
       </c>
-      <c r="C188" s="28" t="s">
+      <c r="C188" s="26" t="s">
         <v>1091</v>
       </c>
       <c r="D188" s="19" t="s">
@@ -20080,7 +20077,7 @@
       <c r="B189" s="18" t="s">
         <v>436</v>
       </c>
-      <c r="C189" s="28" t="s">
+      <c r="C189" s="26" t="s">
         <v>1093</v>
       </c>
       <c r="D189" s="19" t="s">
@@ -20123,7 +20120,7 @@
       <c r="B190" s="18" t="s">
         <v>436</v>
       </c>
-      <c r="C190" s="28" t="s">
+      <c r="C190" s="26" t="s">
         <v>1096</v>
       </c>
       <c r="D190" s="19" t="s">
@@ -20166,7 +20163,7 @@
       <c r="B191" s="18" t="s">
         <v>436</v>
       </c>
-      <c r="C191" s="28" t="s">
+      <c r="C191" s="26" t="s">
         <v>1101</v>
       </c>
       <c r="D191" s="19" t="s">
@@ -20207,7 +20204,7 @@
       <c r="B192" s="18" t="s">
         <v>436</v>
       </c>
-      <c r="C192" s="28" t="s">
+      <c r="C192" s="26" t="s">
         <v>1104</v>
       </c>
       <c r="D192" s="19" t="s">
@@ -20252,7 +20249,7 @@
       <c r="B193" s="19" t="s">
         <v>440</v>
       </c>
-      <c r="C193" s="28" t="s">
+      <c r="C193" s="26" t="s">
         <v>1107</v>
       </c>
       <c r="D193" s="19" t="s">
@@ -20291,7 +20288,7 @@
       <c r="B194" s="19" t="s">
         <v>440</v>
       </c>
-      <c r="C194" s="28" t="s">
+      <c r="C194" s="26" t="s">
         <v>1110</v>
       </c>
       <c r="D194" s="19" t="s">
@@ -20332,7 +20329,7 @@
       <c r="B195" s="19" t="s">
         <v>445</v>
       </c>
-      <c r="C195" s="28" t="s">
+      <c r="C195" s="26" t="s">
         <v>1113</v>
       </c>
       <c r="D195" s="19" t="s">
@@ -20373,7 +20370,7 @@
       <c r="B196" s="19" t="s">
         <v>445</v>
       </c>
-      <c r="C196" s="28" t="s">
+      <c r="C196" s="26" t="s">
         <v>1115</v>
       </c>
       <c r="D196" s="19" t="s">
@@ -20410,7 +20407,7 @@
       <c r="B197" s="19" t="s">
         <v>445</v>
       </c>
-      <c r="C197" s="28" t="s">
+      <c r="C197" s="26" t="s">
         <v>1117</v>
       </c>
       <c r="D197" s="19" t="s">
@@ -20451,7 +20448,7 @@
       <c r="B198" s="19" t="s">
         <v>445</v>
       </c>
-      <c r="C198" s="28" t="s">
+      <c r="C198" s="26" t="s">
         <v>1119</v>
       </c>
       <c r="D198" s="19" t="s">
@@ -20488,7 +20485,7 @@
       <c r="B199" s="19" t="s">
         <v>450</v>
       </c>
-      <c r="C199" s="28" t="s">
+      <c r="C199" s="26" t="s">
         <v>1122</v>
       </c>
       <c r="D199" s="19" t="s">
@@ -20531,7 +20528,7 @@
       <c r="B200" s="19" t="s">
         <v>450</v>
       </c>
-      <c r="C200" s="28" t="s">
+      <c r="C200" s="26" t="s">
         <v>1124</v>
       </c>
       <c r="D200" s="19" t="s">
@@ -20576,7 +20573,7 @@
       <c r="B201" s="19" t="s">
         <v>450</v>
       </c>
-      <c r="C201" s="28" t="s">
+      <c r="C201" s="26" t="s">
         <v>1126</v>
       </c>
       <c r="D201" s="19" t="s">
@@ -20621,7 +20618,7 @@
       <c r="B202" s="19" t="s">
         <v>450</v>
       </c>
-      <c r="C202" s="28" t="s">
+      <c r="C202" s="26" t="s">
         <v>1131</v>
       </c>
       <c r="D202" s="19" t="s">
@@ -20668,7 +20665,7 @@
       <c r="B203" s="19" t="s">
         <v>450</v>
       </c>
-      <c r="C203" s="28" t="s">
+      <c r="C203" s="26" t="s">
         <v>1137</v>
       </c>
       <c r="D203" s="19" t="s">
@@ -20711,7 +20708,7 @@
       <c r="B204" s="19" t="s">
         <v>450</v>
       </c>
-      <c r="C204" s="28" t="s">
+      <c r="C204" s="26" t="s">
         <v>1140</v>
       </c>
       <c r="D204" s="19" t="s">
@@ -20756,7 +20753,7 @@
       <c r="B205" s="19" t="s">
         <v>450</v>
       </c>
-      <c r="C205" s="28" t="s">
+      <c r="C205" s="26" t="s">
         <v>1143</v>
       </c>
       <c r="D205" s="19" t="s">
@@ -20801,7 +20798,7 @@
       <c r="B206" s="19" t="s">
         <v>455</v>
       </c>
-      <c r="C206" s="28" t="s">
+      <c r="C206" s="26" t="s">
         <v>1147</v>
       </c>
       <c r="D206" s="19" t="s">

</xml_diff>